<commit_message>
Email Text To Pay on Prod
</commit_message>
<xml_diff>
--- a/KatalonData/ABPTestData/PaymentsACH.xlsx
+++ b/KatalonData/ABPTestData/PaymentsACH.xlsx
@@ -74,7 +74,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1295" uniqueCount="213">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1335" uniqueCount="218">
   <si>
     <t>Result</t>
   </si>
@@ -954,6 +954,21 @@
   </si>
   <si>
     <t>Wed Mar 11 00:28:09 IST 2026</t>
+  </si>
+  <si>
+    <t>Thu Mar 12 21:04:26 IST 2026</t>
+  </si>
+  <si>
+    <t>Thu Mar 12 21:16:08 IST 2026</t>
+  </si>
+  <si>
+    <t>Thu Mar 12 21:19:26 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Mar 13 00:09:23 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Mar 13 00:16:10 IST 2026</t>
   </si>
 </sst>
 </file>
@@ -3741,7 +3756,7 @@
         <v>10</v>
       </c>
       <c r="B2" t="s">
-        <v>209</v>
+        <v>217</v>
       </c>
       <c r="C2" s="14"/>
       <c r="D2" s="12" t="s">

</xml_diff>